<commit_message>
paper run 2026-10-15 10:01
</commit_message>
<xml_diff>
--- a/reports/2026-10-15.xlsx
+++ b/reports/2026-10-15.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,6 +515,92 @@
       </c>
       <c r="K2" t="n">
         <v>4.9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:41:18.172402+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F3" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="G3" t="n">
+        <v>16.36</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.00181</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>-10.14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-15T07:56:24.132035+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="G4" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.765</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.00125</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>2.8</v>
       </c>
     </row>
   </sheetData>
@@ -528,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,7 +636,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -560,7 +646,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -570,7 +656,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -580,7 +666,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="6">
@@ -590,7 +676,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4.9</v>
+        <v>-2.44</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +686,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4.9</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="8">
@@ -610,7 +696,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>-10.14</v>
       </c>
     </row>
     <row r="9">
@@ -620,7 +706,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>99</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="10">
@@ -630,7 +716,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3329.479999999999</v>
+        <v>3322.139999999999</v>
       </c>
     </row>
     <row r="12">
@@ -681,16 +767,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
-        <v>460.56</v>
+        <v>373.51</v>
       </c>
       <c r="E15" t="n">
-        <v>4.9</v>
+        <v>-2.44</v>
       </c>
     </row>
     <row r="16">
@@ -700,13 +786,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>136.21</v>
+        <v>111.95</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -726,16 +812,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>153.44</v>
+        <v>105.61</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="19">
@@ -745,16 +831,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>147.41</v>
+        <v>2.08</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>-10.14</v>
       </c>
     </row>
     <row r="20">
@@ -764,13 +850,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>295.92</v>
+        <v>377.77</v>
       </c>
       <c r="E20" t="n">
         <v>4.9</v>
@@ -790,13 +876,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D22" t="n">
-        <v>596.77</v>
+        <v>734.36</v>
       </c>
       <c r="E22" t="n">
         <v>4.9</v>
@@ -805,252 +891,278 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-47.83</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2.8</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MAX_PER_WINDOW</t>
+          <t>0.60–0.62</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>300.85</v>
+        <v>-201.07</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>-10.14</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" t="n">
-        <v>136.21</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MAX_PER_WINDOW</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>159.71</v>
+        <v>136.19</v>
       </c>
       <c r="E26" t="n">
-        <v>4.9</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="n">
+        <v>218.06</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" t="n">
+        <v>131.21</v>
+      </c>
+      <c r="E28" t="n">
+        <v>-2.44</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>По активам</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" t="n">
-        <v>4.9</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>2.8</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>15m</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D34" t="n">
+        <v>-10.14</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
         <v>4.9</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" t="n">
-        <v>4.9</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>3</v>
+      </c>
+      <c r="C38" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" t="n">
+        <v>-2.44</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" t="n">
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
         <v>4.9</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>-10.14</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0.20%+</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1060,13 +1172,13 @@
         <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>4.9</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>По направлению</t>
+          <t>По цене входа</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1088,7 +1200,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1099,6 +1211,162 @@
       </c>
       <c r="D46" t="n">
         <v>4.9</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" t="n">
+        <v>-10.14</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" t="n">
+        <v>-10.14</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>0.20%+</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="n">
+        <v>-7.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-10-15 16:38
</commit_message>
<xml_diff>
--- a/reports/2026-10-15.xlsx
+++ b/reports/2026-10-15.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -601,6 +601,264 @@
       </c>
       <c r="K4" t="n">
         <v>2.8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-15T12:27:23.557285+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.779</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.00103</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-15T13:33:52.347235+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F6" t="n">
+        <v>12.37</v>
+      </c>
+      <c r="G6" t="n">
+        <v>19.95</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.00227</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>7.58</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-15T14:18:53.068821+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F7" t="n">
+        <v>41.18</v>
+      </c>
+      <c r="G7" t="n">
+        <v>71</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.00192</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>29.82</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-15T14:26:23.845842+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="G8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.8120000000000001</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.00279</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>-2.85</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-15T15:08:46.559315+00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F9" t="n">
+        <v>164.11</v>
+      </c>
+      <c r="G9" t="n">
+        <v>269.03</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.795</v>
+      </c>
+      <c r="I9" t="n">
+        <v>-0.0023</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>104.92</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-15T16:11:41.309304+00:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="G10" t="n">
+        <v>10</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.00123</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>-5.3</v>
       </c>
     </row>
   </sheetData>
@@ -614,7 +872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -636,7 +894,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -646,7 +904,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -656,7 +914,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -676,7 +934,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-2.44</v>
+        <v>136.33</v>
       </c>
     </row>
     <row r="7">
@@ -686,7 +944,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7.7</v>
+        <v>154.62</v>
       </c>
     </row>
     <row r="8">
@@ -696,7 +954,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-10.14</v>
+        <v>-18.29</v>
       </c>
     </row>
     <row r="9">
@@ -706,7 +964,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.76</v>
+        <v>8.449999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -716,7 +974,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3322.139999999999</v>
+        <v>3460.909999999999</v>
       </c>
     </row>
     <row r="12">
@@ -767,16 +1025,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D15" t="n">
-        <v>373.51</v>
+        <v>132.3</v>
       </c>
       <c r="E15" t="n">
-        <v>-2.44</v>
+        <v>-5.99</v>
       </c>
     </row>
     <row r="16">
@@ -786,16 +1044,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D16" t="n">
-        <v>111.95</v>
+        <v>955.83</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>142.32</v>
       </c>
     </row>
     <row r="17">
@@ -808,164 +1066,164 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>105.61</v>
+        <v>104.92</v>
       </c>
       <c r="E18" t="n">
-        <v>2.8</v>
+        <v>104.92</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D19" t="n">
-        <v>2.08</v>
+        <v>674.23</v>
       </c>
       <c r="E19" t="n">
-        <v>-10.14</v>
+        <v>32.62</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D20" t="n">
-        <v>377.77</v>
+        <v>171.61</v>
       </c>
       <c r="E20" t="n">
-        <v>4.9</v>
+        <v>-3.26</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>10</v>
+      </c>
+      <c r="C21" t="n">
+        <v>6</v>
+      </c>
+      <c r="D21" t="n">
+        <v>137.37</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2.05</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>5</v>
-      </c>
-      <c r="C22" t="n">
-        <v>5</v>
-      </c>
-      <c r="D22" t="n">
-        <v>734.36</v>
-      </c>
-      <c r="E22" t="n">
-        <v>4.9</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D23" t="n">
-        <v>-47.83</v>
+        <v>1094.83</v>
       </c>
       <c r="E23" t="n">
-        <v>2.8</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B24" t="n">
+        <v>6</v>
+      </c>
+      <c r="C24" t="n">
         <v>3</v>
       </c>
-      <c r="C24" t="n">
-        <v>1</v>
-      </c>
       <c r="D24" t="n">
-        <v>-201.07</v>
+        <v>-116.54</v>
       </c>
       <c r="E24" t="n">
-        <v>-10.14</v>
+        <v>29.77</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>6</v>
+      </c>
+      <c r="C25" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" t="n">
+        <v>109.84</v>
+      </c>
+      <c r="E25" t="n">
+        <v>102.36</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MAX_PER_WINDOW</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>3</v>
-      </c>
-      <c r="C26" t="n">
-        <v>2</v>
-      </c>
-      <c r="D26" t="n">
-        <v>136.19</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>MAX_PER_WINDOW</t>
         </is>
       </c>
       <c r="B27" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" t="n">
         <v>4</v>
       </c>
-      <c r="C27" t="n">
-        <v>3</v>
-      </c>
       <c r="D27" t="n">
-        <v>218.06</v>
+        <v>397.91</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -974,233 +1232,246 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>14</v>
+      </c>
+      <c r="C28" t="n">
+        <v>9</v>
+      </c>
+      <c r="D28" t="n">
+        <v>433.98</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B28" t="n">
-        <v>3</v>
-      </c>
-      <c r="C28" t="n">
-        <v>2</v>
-      </c>
-      <c r="D28" t="n">
-        <v>131.21</v>
-      </c>
-      <c r="E28" t="n">
-        <v>-2.44</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="B29" t="n">
+        <v>9</v>
+      </c>
+      <c r="C29" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" t="n">
+        <v>256.24</v>
+      </c>
+      <c r="E29" t="n">
+        <v>136.33</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ETH</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" t="n">
-        <v>2.8</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>-10.14</v>
+        <v>104.92</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35" t="n">
-        <v>4.9</v>
+        <v>32.62</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>4</v>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="n">
+        <v>-3.26</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>По окнам</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>3</v>
-      </c>
-      <c r="C38" t="n">
-        <v>2</v>
-      </c>
-      <c r="D38" t="n">
-        <v>-2.44</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>6</v>
+      </c>
+      <c r="C40" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" t="n">
+        <v>-5.99</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>5m</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D41" t="n">
-        <v>4.9</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" t="n">
-        <v>0</v>
-      </c>
-      <c r="D42" t="n">
-        <v>-10.14</v>
+        <v>142.32</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" t="n">
-        <v>2.8</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>4.9</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>-10.14</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1210,13 +1481,13 @@
         <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>4.9</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1226,147 +1497,281 @@
         <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>2.8</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>1</v>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D48" t="n">
-        <v>-10.14</v>
+        <v>7.58</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>26.97</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>104.92</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>1</v>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D51" t="n">
-        <v>2.8</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>0.15–0.20%</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>1</v>
-      </c>
-      <c r="C52" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" t="n">
-        <v>-10.14</v>
+        <v>-5.3</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0.20%+</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>1</v>
-      </c>
-      <c r="C53" t="n">
-        <v>1</v>
-      </c>
-      <c r="D53" t="n">
-        <v>4.9</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" t="n">
+        <v>4.2</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>3</v>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="n">
+        <v>29.77</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" t="n">
+        <v>102.36</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>2</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" t="n">
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>2</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" t="n">
+        <v>19.68</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>0.20%+</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>4</v>
+      </c>
+      <c r="C62" t="n">
+        <v>3</v>
+      </c>
+      <c r="D62" t="n">
+        <v>114.55</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B56" t="n">
-        <v>1</v>
-      </c>
-      <c r="C56" t="n">
-        <v>1</v>
-      </c>
-      <c r="D56" t="n">
-        <v>4.9</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="B65" t="n">
+        <v>3</v>
+      </c>
+      <c r="C65" t="n">
+        <v>3</v>
+      </c>
+      <c r="D65" t="n">
+        <v>114.42</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B57" t="n">
-        <v>2</v>
-      </c>
-      <c r="C57" t="n">
-        <v>1</v>
-      </c>
-      <c r="D57" t="n">
-        <v>-7.34</v>
+      <c r="B66" t="n">
+        <v>6</v>
+      </c>
+      <c r="C66" t="n">
+        <v>3</v>
+      </c>
+      <c r="D66" t="n">
+        <v>21.91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-10-15 22:18
</commit_message>
<xml_diff>
--- a/reports/2026-10-15.xlsx
+++ b/reports/2026-10-15.xlsx
@@ -1025,13 +1025,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D15" t="n">
-        <v>132.3</v>
+        <v>279.7</v>
       </c>
       <c r="E15" t="n">
         <v>-5.99</v>
@@ -1108,13 +1108,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D20" t="n">
-        <v>171.61</v>
+        <v>319.01</v>
       </c>
       <c r="E20" t="n">
         <v>-3.26</v>
@@ -1153,13 +1153,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C23" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D23" t="n">
-        <v>1094.83</v>
+        <v>1242.23</v>
       </c>
       <c r="E23" t="n">
         <v>4.2</v>
@@ -1236,13 +1236,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C28" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D28" t="n">
-        <v>433.98</v>
+        <v>581.38</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>

</xml_diff>